<commit_message>
Farmácia: item com fabricante nunca fica OUTRA MARCA (nome comercial, nome do produto como genérico ou nome do fabricante)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ymBuSrNzAQRN5kGJoFo1p
</commit_message>
<xml_diff>
--- a/classificador/dados/vitamina_mineral_500_classificado.xlsx
+++ b/classificador/dados/vitamina_mineral_500_classificado.xlsx
@@ -5908,25 +5908,25 @@
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>7898994538714</v>
+        <v>1286508384821</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>SUPL ALIM 1000MG 1UN (MXR)</t>
+          <t>SUPL ALIM ALIMENTA DESINCHA 500MG 90CPS (ALI)</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>MAXINUTRI</t>
+          <t>ALIMENTA</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>OUTRA MARCA</t>
+          <t>ALIMENTA ALI</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -5950,31 +5950,31 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>CODIGO INTERNO</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>7898605844258</v>
+        <v>606529303372</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SUPL ALIM 1UN (BAG)</t>
+          <t>SUPL ALIM ALQUIMIA DA SAUDE DETOX 600MG 90CPS (ALQ)</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>BAGO</t>
+          <t>ALQUIMIA</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>OUTRA MARCA</t>
+          <t>ALQUIMIA DA SAUDE ALQ</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -5998,31 +5998,31 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>JARDINAGEM</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>1286508384821</v>
+        <v>7899468501210</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>SUPL ALIM ALIMENTA DESINCHA 500MG 90CPS (ALI)</t>
+          <t>SUPL ALIM APISNUTRI OLEO DE COCO EXTRA 1000.0MG 60G (APN)</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ALIMENTA</t>
+          <t>APISNUTRI</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>ALIMENTA ALI</t>
+          <t>APISNUTRI APN</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -6046,31 +6046,31 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>CODIGO INTERNO</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>606529303372</v>
+        <v>7898700720266</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>SUPL ALIM ALQUIMIA DA SAUDE DETOX 600MG 90CPS (ALQ)</t>
+          <t>SUPL ALIM ATLANTICA HEALTH CALM 30CPRS (ATA)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ALQUIMIA</t>
+          <t>ATLANTICA HEALTH</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>ALQUIMIA DA SAUDE ALQ</t>
+          <t>ATLANTICA HEALTH ATA</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -6094,31 +6094,31 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>VESTUARIO</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>7899468501210</v>
+        <v>7898946434019</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SUPL ALIM APISNUTRI OLEO DE COCO EXTRA 1000.0MG 60G (APN)</t>
+          <t>SUPL ALIM B WELL LUTEINA CAPSUALAS 10MG 30UN (RDF)</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>APISNUTRI</t>
+          <t>RAIA DROGASIL SA</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>APISNUTRI APN</t>
+          <t>B WELL RDF</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -6142,31 +6142,31 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>PEQUENO DOMESTICO</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>7898700720266</v>
+        <v>7897535410595</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SUPL ALIM ATLANTICA HEALTH CALM 30CPRS (ATA)</t>
+          <t>SUPL ALIM BARBARA BERINJELA 500MG 50CPS (MAR)</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ATLANTICA HEALTH</t>
+          <t>MARCK BEBIDAS</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ATLANTICA HEALTH ATA</t>
+          <t>BARBARA MAR</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -6190,31 +6190,31 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>VESTUARIO</t>
+          <t>CACHACA</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>7898946434019</v>
+        <v>7898932877035</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SUPL ALIM B WELL LUTEINA CAPSUALAS 10MG 30UN (RDF)</t>
+          <t>SUPL ALIM BELVCAPS BERINJELA NATURA 250MG 60CPS (BLV)</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>RAIA DROGASIL SA</t>
+          <t>BELV CAPS</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>B WELL RDF</t>
+          <t>BELVCAPS BLV</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -6238,31 +6238,31 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>PEQUENO DOMESTICO</t>
+          <t>CACHACA</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>7897535410595</v>
+        <v>7898932877585</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>SUPL ALIM BARBARA BERINJELA 500MG 50CPS (MAR)</t>
+          <t>SUPL ALIM BELVCAPS CAFEINA 500MG 60CPS (BLV)</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>MARCK BEBIDAS</t>
+          <t>BELV CAPS</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>BARBARA MAR</t>
+          <t>BELVCAPS BLV</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -6286,27 +6286,27 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>CACHACA</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>7898932877035</v>
+        <v>7898605843374</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>SUPL ALIM BELVCAPS BERINJELA NATURA 250MG 60CPS (BLV)</t>
+          <t>SUPL ALIM BIOTINA 60UN (BAG)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>BELV CAPS</t>
+          <t>BAGO</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>BELVCAPS BLV</t>
+          <t>BIOTINA BAG</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -6334,27 +6334,27 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>CACHACA</t>
+          <t>BRINQUEDO</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>7898932877585</v>
+        <v>7898556034524</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>SUPL ALIM BELVCAPS CAFEINA 500MG 60CPS (BLV)</t>
+          <t>SUPL ALIM BORG MAGNESIO 500MG 60CPS (ASS)</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>BELV CAPS</t>
+          <t>ASSIFARMA</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>BELVCAPS BLV</t>
+          <t>BORG ASS</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -6388,21 +6388,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>7898605843374</v>
+        <v>7898929983121</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>SUPL ALIM BIOTINA 60UN (BAG)</t>
+          <t>SUPL ALIM CAFE VERDE 500.0MG 60CPS (MUW)</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>BAGO</t>
+          <t>MUWIZ</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>BIOTINA BAG</t>
+          <t>CAFE VERDE MUW</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -6430,31 +6430,31 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>BRINQUEDO</t>
+          <t>CAFE</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>7898556034524</v>
+        <v>7898374654614</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SUPL ALIM BORG MAGNESIO 500MG 60CPS (ASS)</t>
+          <t>SUPL ALIM CARDIOSETYL LIQUIDO 120ML</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ASSIFARMA</t>
+          <t>OUTRO FABRICANTE</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>BORG ASS</t>
+          <t>OUTRA MARCA</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -6471,6 +6471,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I123" s="4" t="inlineStr">
+        <is>
+          <t>SEM FABRICANTE</t>
+        </is>
+      </c>
       <c r="K123" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6478,31 +6483,31 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>ACESSORIO PARA COSMETICA</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>7898929983121</v>
+        <v>7898636648863</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>SUPL ALIM CAFE VERDE 500.0MG 60CPS (MUW)</t>
+          <t>SUPL ALIM CENTRO FLEX CURCUMA MIX GOTAS ABACAXI 30ML (ARO)</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>MUWIZ</t>
+          <t>AROMA BEM ESTAR IND E COM DE PROD NATURAIS</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>CAFE VERDE MUW</t>
+          <t>CENTRO FLEX ARO</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -6526,17 +6531,17 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>CAFE</t>
+          <t>GRAO OUTROS</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>7898374654614</v>
+        <v>7896201801279</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>SUPL ALIM CARDIOSETYL LIQUIDO 120ML</t>
+          <t>SUPL ALIM CHA VERDE 60CPRS</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -6550,7 +6555,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -6579,31 +6584,31 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>ACESSORIO PARA COSMETICA</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>7898636648863</v>
+        <v>7908730202134</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>SUPL ALIM CENTRO FLEX CURCUMA MIX GOTAS ABACAXI 30ML (ARO)</t>
+          <t>SUPL ALIM CIMEVITAN TESTO MAM SIDNEY 60CPRS (ULT)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>AROMA BEM ESTAR IND E COM DE PROD NATURAIS</t>
+          <t>ULTRAFARMA</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>CENTRO FLEX ARO</t>
+          <t>CIMEVITAN ULT</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -6627,31 +6632,31 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>GRAO OUTROS</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>7896201801279</v>
+        <v>7896004718088</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>SUPL ALIM CHA VERDE 60CPRS</t>
+          <t>SUPL ALIM COBAGLOBAL XAROPE 100ML (SLA)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>SOLARIS PHARMA</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>OUTRA MARCA</t>
+          <t>COBAGLOBAL SLA</t>
         </is>
       </c>
       <c r="E127" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -6668,11 +6673,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I127" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
-        </is>
-      </c>
       <c r="K127" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6680,27 +6680,27 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>CERVEJA</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
-        <v>7908730202134</v>
+        <v>7898947407531</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SUPL ALIM CIMEVITAN TESTO MAM SIDNEY 60CPRS (ULT)</t>
+          <t>SUPL ALIM COQ 10 COENZYME Q10 VITAMINLIFE 50MG 60CPS (VTF)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ULTRAFARMA</t>
+          <t>VITAFOR</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>CIMEVITAN ULT</t>
+          <t>COQ 10 VTF</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -6728,31 +6728,31 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>LEGUME</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
-        <v>7896004718088</v>
+        <v>631911666827</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SUPL ALIM COBAGLOBAL XAROPE 100ML (SLA)</t>
+          <t>SUPL ALIM COQ 10 LIQUID FRUT 225ML (TRU)</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>SOLARIS PHARMA</t>
+          <t>TRUE SOURCE</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>COBAGLOBAL SLA</t>
+          <t>COQ 10 TRU</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>100</v>
+        <v>225</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -6776,17 +6776,17 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>CERVEJA</t>
+          <t>TRATAMENTO CAPILAR</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
-        <v>7898947407531</v>
+        <v>7898665430064</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SUPL ALIM COQ 10 COENZYME Q10 VITAMINLIFE 50MG 60CPS (VTF)</t>
+          <t>SUPL ALIM CURC VITAF 1000MG 60CPS (VTF)</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -6796,7 +6796,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>COQ 10 VTF</t>
+          <t>CURC VTF</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -6824,31 +6824,31 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>LEGUME</t>
+          <t>PEIXE</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
-        <v>631911666827</v>
+        <v>7898605844258</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>SUPL ALIM COQ 10 LIQUID FRUT 225ML (TRU)</t>
+          <t>SUPL ALIM DESCRICAO 1UN (BAG)</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>TRUE SOURCE</t>
+          <t>BAGO</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>COQ 10 TRU</t>
+          <t>DESCRICAO BAG</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>225</v>
+        <v>1</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -6865,6 +6865,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I131" s="4" t="inlineStr">
+        <is>
+          <t>CRIAR MARCA</t>
+        </is>
+      </c>
       <c r="K131" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6872,27 +6877,27 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>TRATAMENTO CAPILAR</t>
+          <t>JARDINAGEM</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
-        <v>7898665430064</v>
+        <v>7898684480903</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>SUPL ALIM CURC VITAF 1000MG 60CPS (VTF)</t>
+          <t>SUPL ALIM DESINCHA NEURO BOOST 60CPS</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>VITAFOR</t>
+          <t>OUTRO FABRICANTE</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>CURC VTF</t>
+          <t>OUTRA MARCA</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -6913,6 +6918,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I132" s="4" t="inlineStr">
+        <is>
+          <t>SEM FABRICANTE</t>
+        </is>
+      </c>
       <c r="K132" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6920,27 +6930,27 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>PEIXE</t>
+          <t>ACESSORIO CASA</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
-        <v>7898684480903</v>
+        <v>7908228801344</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>SUPL ALIM DESINCHA NEURO BOOST 60CPS</t>
+          <t>SUPL ALIM DR GOOD VITAMINA 60UN (SNC)</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>AURAQUIMICA</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>OUTRA MARCA</t>
+          <t>DR GOOD SNC</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -6961,11 +6971,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I133" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
-        </is>
-      </c>
       <c r="K133" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6973,17 +6978,17 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>ACESSORIO CASA</t>
+          <t>VERDURA</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
-        <v>7908228801344</v>
+        <v>7898946434996</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>SUPL ALIM DR GOOD VITAMINA 60UN (SNC)</t>
+          <t>SUPL ALIM DROGASIL CAFEINA 1UN (RDF)</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -6993,11 +6998,11 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>DR GOOD SNC</t>
+          <t>DROGASIL RDF</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -7021,17 +7026,17 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>VERDURA</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
-        <v>7898946434996</v>
+        <v>7891066007583</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>SUPL ALIM DROGASIL CAFEINA 1UN (RDF)</t>
+          <t>SUPL ALIM DROGASIL COENZ Q10 30UN (RDF)</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -7045,7 +7050,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -7075,11 +7080,11 @@
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>7891066007583</v>
+        <v>7891066007606</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SUPL ALIM DROGASIL COENZ Q10 30UN (RDF)</t>
+          <t>SUPL ALIM DROGASIL COENZ Q10 60UN (RDF)</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -7093,7 +7098,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -7123,11 +7128,11 @@
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>7891066007606</v>
+        <v>7891066002939</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SUPL ALIM DROGASIL COENZ Q10 60UN (RDF)</t>
+          <t>SUPL ALIM DROGASIL VIT 1UN (RDF)</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7141,7 +7146,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -7171,11 +7176,11 @@
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
-        <v>7891066002939</v>
+        <v>7891066005206</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>SUPL ALIM DROGASIL VIT 1UN (RDF)</t>
+          <t>SUPL ALIM DROGASIL VIT CZINC 30UN (RDF)</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7189,7 +7194,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -7219,11 +7224,11 @@
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>7891066005206</v>
+        <v>7891066005183</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>SUPL ALIM DROGASIL VIT CZINC 30UN (RDF)</t>
+          <t>SUPL ALIM DROGASIL VITAMINA C ZINCO 10CPRS (RDF)</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7237,7 +7242,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -7267,25 +7272,25 @@
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
-        <v>7891066005183</v>
+        <v>7898958836801</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>SUPL ALIM DROGASIL VITAMINA C ZINCO 10CPRS (RDF)</t>
+          <t>SUPL ALIM DUOM OLEO ALHO DESODORIZADO 500.0MG 60CPS (DMO)</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>AURAQUIMICA</t>
+          <t>DUOM</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>DROGASIL RDF</t>
+          <t>DUOM DMO</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -7309,27 +7314,27 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
-        <v>7898958836801</v>
+        <v>7898215158943</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>SUPL ALIM DUOM OLEO ALHO DESODORIZADO 500.0MG 60CPS (DMO)</t>
+          <t>SUPL ALIM EMANA GUMMY VINAGRE DE MACA 60UN (EMN)</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>DUOM</t>
+          <t>EMANA</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>DUOM DMO</t>
+          <t>EMANA EMN</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -7357,31 +7362,31 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
-        <v>7898215158943</v>
+        <v>7899547018578</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>SUPL ALIM EMANA GUMMY VINAGRE DE MACA 60UN (EMN)</t>
+          <t>SUPL ALIM ENERGY CAFEX EXTRA FORTE 420MG 4UN (CAT)</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>EMANA</t>
+          <t>ENERGY UP</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>EMANA EMN</t>
+          <t>ENERGY CAT</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -7405,31 +7410,31 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>ENERGETICO</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
-        <v>7899547018578</v>
+        <v>7895537068226</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>SUPL ALIM ENERGY CAFEX EXTRA FORTE 420MG 4UN (CAT)</t>
+          <t>SUPL ALIM ESSENCIAL VINAGRE DE MACA 500.0MG 60CPS (BIO)</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ENERGY UP</t>
+          <t>BIOLAB</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ENERGY CAT</t>
+          <t>ESSENCIAL BIO</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -7453,27 +7458,27 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>ENERGETICO</t>
+          <t>VINAGRE</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
-        <v>7895537068226</v>
+        <v>7898638342547</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>SUPL ALIM ESSENCIAL VINAGRE DE MACA 500.0MG 60CPS (BIO)</t>
+          <t>SUPL ALIM EUROFITO OMEGA 3 60CPS (EUF)</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>BIOLAB</t>
+          <t>EUROFITO</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>ESSENCIAL BIO</t>
+          <t>EUROFITO EUF</t>
         </is>
       </c>
       <c r="E144" t="n">
@@ -7501,27 +7506,27 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>VINAGRE</t>
+          <t>HIDRAULICA</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
-        <v>7898638342547</v>
+        <v>7898948981030</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>SUPL ALIM EUROFITO OMEGA 3 60CPS (EUF)</t>
+          <t>SUPL ALIM FITO NATURAIS BERINJELA 500MG 60CPS (FIR)</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>EUROFITO</t>
+          <t>FITO NATURAIS</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>EUROFITO EUF</t>
+          <t>FITO NATURAIS FIR</t>
         </is>
       </c>
       <c r="E145" t="n">
@@ -7549,31 +7554,31 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>HIDRAULICA</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
-        <v>7898948981030</v>
+        <v>7898583663674</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>SUPL ALIM FITO NATURAIS BERINJELA 500MG 60CPS (FIR)</t>
+          <t>SUPL ALIM FITOWAY OLEO COCO 120CPS (FIW)</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>FITO NATURAIS</t>
+          <t>FITOWAY</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>FITO NATURAIS FIR</t>
+          <t>FITOWAY FIW</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F146" t="inlineStr">
         <is>
@@ -7597,31 +7602,31 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n">
-        <v>7898583663674</v>
+        <v>7896321021502</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>SUPL ALIM FITOWAY OLEO COCO 120CPS (FIW)</t>
+          <t>SUPL ALIM FLOFARMA FLORESTAL DROPS VIT CPT 45.0MG 160G (FLO)</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>FITOWAY</t>
+          <t>FLOFARMA</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>FITOWAY FIW</t>
+          <t>FLOFARMA FLO</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -7645,31 +7650,31 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>CHOCOLATE</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
-        <v>7896321021502</v>
+        <v>7896321022035</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>SUPL ALIM FLOFARMA FLORESTAL DROPS VIT CPT 45.0MG 160G (FLO)</t>
+          <t>SUPL ALIM FLOPI KIDS PASTILHA VITAMINA C B7 14.4G (FLO)</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>FLOFARMA</t>
+          <t>FLORESTAL</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>FLOFARMA FLO</t>
+          <t>FLOPI KIDS FLO</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>160</v>
+        <v>14.4</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
@@ -7693,17 +7698,17 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>CHOCOLATE</t>
+          <t>BALA E PIRULITO</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n">
-        <v>7896321022035</v>
+        <v>7896321022042</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>SUPL ALIM FLOPI KIDS PASTILHA VITAMINA C B7 14.4G (FLO)</t>
+          <t>SUPL ALIM FLOPI KIDS PASTILHA VITAMINA D 14.4G (FLO)</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7747,11 +7752,11 @@
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
-        <v>7896321022042</v>
+        <v>7896321022066</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>SUPL ALIM FLOPI KIDS PASTILHA VITAMINA D 14.4G (FLO)</t>
+          <t>SUPL ALIM FLOPI KIDS PASTILHA ZINCO MENTA 14.4G (FLO)</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -7795,11 +7800,11 @@
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
-        <v>7896321022066</v>
+        <v>7896321017086</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>SUPL ALIM FLOPI KIDS PASTILHA ZINCO MENTA 14.4G (FLO)</t>
+          <t>SUPL ALIM FLOPI KIDS PICOLINATO CROMO 60G (FLO)</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -7813,7 +7818,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>14.4</v>
+        <v>60</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
@@ -7837,31 +7842,31 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>BALA E PIRULITO</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
-        <v>7896321017086</v>
+        <v>7894911865413</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>SUPL ALIM FLOPI KIDS PICOLINATO CROMO 60G (FLO)</t>
+          <t>SUPL ALIM GOJI BERRY SECA BARRIGA 90CPS (BES)</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>FLORESTAL</t>
+          <t>BESINS HEALTHCARE</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>FLOPI KIDS FLO</t>
+          <t>GOJI BERRY BES</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
@@ -7885,31 +7890,31 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>PRODUTOS ORIENTAIS</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n">
-        <v>7894911865413</v>
+        <v>7896550500038</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>SUPL ALIM GOJI BERRY SECA BARRIGA 90CPS (BES)</t>
+          <t>SUPL ALIM GUARANA 50CPS (DOC)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>BESINS HEALTHCARE</t>
+          <t>DOCES MACHADO</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>GOJI BERRY BES</t>
+          <t>GUARANA DOC</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
@@ -7933,31 +7938,31 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>PRODUTOS ORIENTAIS</t>
+          <t>GUARANA EM PO</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
-        <v>7896550500038</v>
+        <v>7898949730682</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>SUPL ALIM GUARANA 50CPS (DOC)</t>
+          <t>SUPL ALIM GUARANA LIPIX PLUS 120X1KG (VTF)</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>DOCES MACHADO</t>
+          <t>VITAFOR</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>GUARANA DOC</t>
+          <t>GUARANA VTF</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>50</v>
+        <v>120000</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -7981,31 +7986,31 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>GUARANA EM PO</t>
+          <t>PEQUENO DOMESTICO</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n">
-        <v>7898949730682</v>
+        <v>7898615893758</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>SUPL ALIM GUARANA LIPIX PLUS 120X1KG (VTF)</t>
+          <t>SUPL ALIM HIALURE GOLD 30ML (LAS)</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>VITAFOR</t>
+          <t>LA SAN DAY</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>GUARANA VTF</t>
+          <t>HIALURE GOLD LAS</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>120000</v>
+        <v>30</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -8029,27 +8034,27 @@
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>PEQUENO DOMESTICO</t>
+          <t>TRATAMENTO FACIAL</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
-        <v>7898615893758</v>
+        <v>7898656162394</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>SUPL ALIM HIALURE GOLD 30ML (LAS)</t>
+          <t>SUPL ALIM IMUNO 30CPS (BMF)</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>LA SAN DAY</t>
+          <t>BMF VIT</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>HIALURE GOLD LAS</t>
+          <t>BMF BMF</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -8077,31 +8082,31 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>TRATAMENTO FACIAL</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
-        <v>7898656162394</v>
+        <v>7898636861071</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>SUPL ALIM IMUNO 30CPS (BMF)</t>
+          <t>SUPL ALIM JIANG HUANG MTC 700.0MG 120CPS</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>BMF VIT</t>
+          <t>OUTRO FABRICANTE</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>BMF BMF</t>
+          <t>JIANG HUANG</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -8118,6 +8123,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I157" s="4" t="inlineStr">
+        <is>
+          <t>SEM FABRICANTE</t>
+        </is>
+      </c>
       <c r="K157" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -8125,31 +8135,31 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>TEMPERO SECO</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n">
-        <v>7898636861071</v>
+        <v>7898379442186</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>SUPL ALIM JIANG HUANG MTC 700.0MG 120CPS</t>
+          <t>SUPL ALIM JP PEREIRA OLEO PEIERA 1000MG 60CPRS (JPP)</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>JP PEREIRA</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>JIANG HUANG</t>
+          <t>JP PEREIRA JPP</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -8166,11 +8176,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I158" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
-        </is>
-      </c>
       <c r="K158" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -8178,27 +8183,27 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>TEMPERO SECO</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n">
-        <v>7898379442186</v>
+        <v>7898538353070</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>SUPL ALIM JP PEREIRA OLEO PEIERA 1000MG 60CPRS (JPP)</t>
+          <t>SUPL ALIM KAMPO DE ERVAS OLEO COCO DERVAS 60G (KAM)</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>JP PEREIRA</t>
+          <t>KAMPO DE ERVAS</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>JP PEREIRA JPP</t>
+          <t>KAMPO DE ERVAS KAM</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -8232,11 +8237,11 @@
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
-        <v>7898538353070</v>
+        <v>7898538351021</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>SUPL ALIM KAMPO DE ERVAS OLEO COCO DERVAS 60G (KAM)</t>
+          <t>SUPL ALIM KAMPO DE ERVAS OLEO PEIX 60X1G (KAM)</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8280,21 +8285,21 @@
     </row>
     <row r="161">
       <c r="A161" s="2" t="n">
-        <v>7898538351021</v>
+        <v>40232912108</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>SUPL ALIM KAMPO DE ERVAS OLEO PEIX 60X1G (KAM)</t>
+          <t>SUPL ALIM KRILL OLEO DE ESSENT 500MG 60G (ESS)</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>KAMPO DE ERVAS</t>
+          <t>ESSENTIAL NUTRITION</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>KAMPO DE ERVAS KAM</t>
+          <t>KRILL ESS</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -8322,27 +8327,27 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n">
-        <v>40232912108</v>
+        <v>7898303260374</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>SUPL ALIM KRILL OLEO DE ESSENT 500MG 60G (ESS)</t>
+          <t>SUPL ALIM LIFE CHA VERDE NATURAL 500MG 60CPS (HMD)</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>ESSENTIAL NUTRITION</t>
+          <t>HERBAMED</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>KRILL ESS</t>
+          <t>LIFE HMD</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -8370,31 +8375,31 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n">
-        <v>7898303260374</v>
+        <v>7908733202964</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>SUPL ALIM LIFE CHA VERDE NATURAL 500MG 60CPS (HMD)</t>
+          <t>SUPL ALIM LINO VITALEY NUTRI PLUS 120UN (CAR)</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>HERBAMED</t>
+          <t>CARVAO LINO</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>LIFE HMD</t>
+          <t>LINO CAR</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F163" t="inlineStr">
         <is>
@@ -8418,31 +8423,31 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>TRATAMENTO CAPILAR</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n">
-        <v>7908733202964</v>
+        <v>7899594200520</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>SUPL ALIM LINO VITALEY NUTRI PLUS 120UN (CAR)</t>
+          <t>SUPL ALIM MACA PERU SEMPR 1UN</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>CARVAO LINO</t>
+          <t>OUTRO FABRICANTE</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>LINO CAR</t>
+          <t>OUTRA MARCA</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
@@ -8459,6 +8464,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I164" s="4" t="inlineStr">
+        <is>
+          <t>SEM FABRICANTE</t>
+        </is>
+      </c>
       <c r="K164" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -8466,31 +8476,31 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>TRATAMENTO CAPILAR</t>
+          <t>ACUCAR</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n">
-        <v>7899594200520</v>
+        <v>7898744351464</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>SUPL ALIM MACA PERU SEMPR 1UN</t>
+          <t>SUPL ALIM MACA PERUANA NEGRA 500MG 60CPS (VAA)</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>VITTALIFE</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>OUTRA MARCA</t>
+          <t>MACA PERUANA VAA</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F165" t="inlineStr">
         <is>
@@ -8507,11 +8517,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I165" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
-        </is>
-      </c>
       <c r="K165" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -8519,31 +8524,31 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>ACUCAR</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n">
-        <v>7898744351464</v>
+        <v>7898958836702</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>SUPL ALIM MACA PERUANA NEGRA 500MG 60CPS (VAA)</t>
+          <t>SUPL ALIM MALTTA OLEO DE ALHO 500MG 120CPS (DMO)</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>VITTALIFE</t>
+          <t>DUOM</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>MACA PERUANA VAA</t>
+          <t>MALTTA DMO</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
@@ -8567,27 +8572,27 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n">
-        <v>7898958836702</v>
+        <v>7898185267355</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>SUPL ALIM MALTTA OLEO DE ALHO 500MG 120CPS (DMO)</t>
+          <t>SUPL ALIM MEDINAL OLEO DE CARTAMO 1000MG 120CPS (MDN)</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>DUOM</t>
+          <t>MEDINAL</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>MALTTA DMO</t>
+          <t>MEDINAL MDN</t>
         </is>
       </c>
       <c r="E167" t="n">
@@ -8621,25 +8626,25 @@
     </row>
     <row r="168">
       <c r="A168" s="2" t="n">
-        <v>7898185267355</v>
+        <v>7898941401887</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>SUPL ALIM MEDINAL OLEO DE CARTAMO 1000MG 120CPS (MDN)</t>
+          <t>SUPL ALIM MIX NUTRI TESTO MACA 500MG 30CPS (PER)</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>MEDINAL</t>
+          <t>MIX NUTRI</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>MEDINAL MDN</t>
+          <t>MIX NUTRI PER</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="F168" t="inlineStr">
         <is>
@@ -8663,17 +8668,17 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>ACESSORIO COZINHA</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n">
-        <v>7898941401887</v>
+        <v>7898941401979</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>SUPL ALIM MIX NUTRI TESTO MACA 500MG 30CPS (PER)</t>
+          <t>SUPL ALIM MIX NUTRI ZMA 500MG 1UN (MIN)</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -8683,11 +8688,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>MIX NUTRI PER</t>
+          <t>MIX NUTRI MIN</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
@@ -8711,31 +8716,31 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>ACESSORIO COZINHA</t>
+          <t>ACESSORIO PARA CAMPING</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n">
-        <v>7898941401979</v>
+        <v>609963002092</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>SUPL ALIM MIX NUTRI ZMA 500MG 1UN (MIN)</t>
+          <t>SUPL ALIM MUKE OMEGA 3 3UN (MAI)</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>MIX NUTRI</t>
+          <t>MAIS MU</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>MIX NUTRI MIN</t>
+          <t>MUKE MAI</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F170" t="inlineStr">
         <is>
@@ -8759,31 +8764,31 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>ACESSORIO PARA CAMPING</t>
+          <t>TEMPERO SECO</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">
-        <v>609963002092</v>
+        <v>7898589722481</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>SUPL ALIM MUKE OMEGA 3 3UN (MAI)</t>
+          <t>SUPL ALIM NATIVA VINAGRE DE MACA 500MG 60CPS (FLN)</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>MAIS MU</t>
+          <t>FLORA NATIVA DO BRASIL</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>MUKE MAI</t>
+          <t>NATIVA FLN</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="F171" t="inlineStr">
         <is>
@@ -8807,31 +8812,31 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>TEMPERO SECO</t>
+          <t>VINAGRE</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n">
-        <v>7898589722481</v>
+        <v>7891066008818</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>SUPL ALIM NATIVA VINAGRE DE MACA 500MG 60CPS (FLN)</t>
+          <t>SUPL ALIM NATZ CRANBERRY EXTRATO VITAMINA C 90CPS (RDF)</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>FLORA NATIVA DO BRASIL</t>
+          <t>MIDWAY LABS</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>NATIVA FLN</t>
+          <t>NATZ RDF</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F172" t="inlineStr">
         <is>
@@ -8855,31 +8860,31 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>VINAGRE</t>
+          <t>PET ACESSORIO</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n">
-        <v>7891066008818</v>
+        <v>7898330228064</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>SUPL ALIM NATZ CRANBERRY EXTRATO VITAMINA C 90CPS (RDF)</t>
+          <t>SUPL ALIM NAYNA CHA ERVAS 525MG 60CPS (KAT)</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>MIDWAY LABS</t>
+          <t>KATIGUA</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>NATZ RDF</t>
+          <t>NAYNA KAT</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F173" t="inlineStr">
         <is>
@@ -8903,31 +8908,31 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>PET ACESSORIO</t>
+          <t>TEMPERO SECO</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
-        <v>7898330228064</v>
+        <v>7897356000531</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>SUPL ALIM NAYNA CHA ERVAS 525MG 60CPS (KAT)</t>
+          <t>SUPL ALIM NECTAR PLUS OLEO DE CHIA 500MG 80CPS (NEA)</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>KATIGUA</t>
+          <t>NECTAR PLUS</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>NAYNA KAT</t>
+          <t>NECTAR PLUS NEA</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -8951,31 +8956,31 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>TEMPERO SECO</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n">
-        <v>7897356000531</v>
+        <v>7899010020244</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>SUPL ALIM NECTAR PLUS OLEO DE CHIA 500MG 80CPS (NEA)</t>
+          <t>SUPL ALIM NUTRIGOLD GELEIA REAL PRO AGARICUS 180CPRS (NTO)</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>NECTAR PLUS</t>
+          <t>NUTRIGOLD DO BRASIL</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>NECTAR PLUS NEA</t>
+          <t>NUTRIGOLD NTO</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>80</v>
+        <v>180</v>
       </c>
       <c r="F175" t="inlineStr">
         <is>
@@ -8999,31 +9004,31 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>GELEIA OUTROS</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
-        <v>7899010020244</v>
+        <v>7908879600389</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>SUPL ALIM NUTRIGOLD GELEIA REAL PRO AGARICUS 180CPRS (NTO)</t>
+          <t>SUPL ALIM NUTRYE VINALLI DE MACA GOMA MAST 60UN (GUM)</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>NUTRIGOLD DO BRASIL</t>
+          <t>ALQUIMIA</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>NUTRIGOLD NTO</t>
+          <t>NUTRYE GUM</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="F176" t="inlineStr">
         <is>
@@ -9047,31 +9052,31 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>GELEIA OUTROS</t>
+          <t>VINAGRE</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n">
-        <v>7908879600389</v>
+        <v>7898927437459</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>SUPL ALIM NUTRYE VINALLI DE MACA GOMA MAST 60UN (GUM)</t>
+          <t>SUPL ALIM NUTRYERVAS CHA VERDE SOLUVEL 350MG 350G (MXR)</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>ALQUIMIA</t>
+          <t>MAXINUTRI</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>NUTRYE GUM</t>
+          <t>NUTRYERVAS MXR</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>60</v>
+        <v>350</v>
       </c>
       <c r="F177" t="inlineStr">
         <is>
@@ -9095,31 +9100,31 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>VINAGRE</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
-        <v>7898927437459</v>
+        <v>7899620912540</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>SUPL ALIM NUTRYERVAS CHA VERDE SOLUVEL 350MG 350G (MXR)</t>
+          <t>SUPL ALIM OLEO ALHO 250MG 60CPRS (GLO)</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>MAXINUTRI</t>
+          <t>LABORATORIO GLOBO</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>NUTRYERVAS MXR</t>
+          <t>OLEO ALHO GLO</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>350</v>
+        <v>60</v>
       </c>
       <c r="F178" t="inlineStr">
         <is>
@@ -9136,6 +9141,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I178" s="4" t="inlineStr">
+        <is>
+          <t>CRIAR MARCA</t>
+        </is>
+      </c>
       <c r="K178" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -9143,22 +9153,22 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
-        <v>7899620912540</v>
+        <v>7898375670057</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>SUPL ALIM OLEO DE ALHO 250MG 60CPRS (GLO)</t>
+          <t>SUPL ALIM OLEO DE CARTAMO 1UN</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO</t>
+          <t>OUTRO FABRICANTE</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -9167,7 +9177,7 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -9182,6 +9192,11 @@
       <c r="H179" t="inlineStr">
         <is>
           <t>Sem indícios de CI</t>
+        </is>
+      </c>
+      <c r="I179" s="4" t="inlineStr">
+        <is>
+          <t>SEM FABRICANTE</t>
         </is>
       </c>
       <c r="K179" s="3" t="inlineStr">
@@ -9197,11 +9212,11 @@
     </row>
     <row r="180">
       <c r="A180" s="2" t="n">
-        <v>7898375670057</v>
+        <v>7898334339018</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>SUPL ALIM OLEO DE CARTAMO 1UN</t>
+          <t>SUPL ALIM OLEO DE CHIA CARTAMO 60CPS</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -9215,7 +9230,7 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F180" t="inlineStr">
         <is>
@@ -9250,11 +9265,11 @@
     </row>
     <row r="181">
       <c r="A181" s="2" t="n">
-        <v>7898334339018</v>
+        <v>7898197933507</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>SUPL ALIM OLEO DE CHIA CARTAMO 60CPS</t>
+          <t>SUPL ALIM OLEO DE SEMENTE DE ABOBORA 60UN</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -9303,11 +9318,11 @@
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
-        <v>7898197933507</v>
+        <v>7899869700458</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>SUPL ALIM OLEO DE SEMENTE DE ABOBORA 60UN</t>
+          <t>SUPL ALIM OLEO GOLD GREEM CART COCO 60CPS</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -9356,21 +9371,21 @@
     </row>
     <row r="183">
       <c r="A183" s="2" t="n">
-        <v>7899869700458</v>
+        <v>7898593054622</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>SUPL ALIM OLEO GOLD GREEM CART COCO 60CPS</t>
+          <t>SUPL ALIM OMEGA 3 AAZ MXN 60CPS (MXR)</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>MAXINUTRI</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>OUTRA MARCA</t>
+          <t>OMEGA 3 MXR</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -9391,11 +9406,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I183" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
-        </is>
-      </c>
       <c r="K183" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -9403,31 +9413,31 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>FINALIZADOR CAPILAR</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
-        <v>7898593054622</v>
+        <v>7898961206721</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>SUPL ALIM OMEGA 3 AAZ MXN 60CPS (MXR)</t>
+          <t>SUPL ALIM OMEGA 3 HYPERNA 1UN (VDO)</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>MAXINUTRI</t>
+          <t>VIDORA</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>OMEGA 3 MXR</t>
+          <t>OMEGA 3 VDO</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F184" t="inlineStr">
         <is>
@@ -9451,17 +9461,17 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>FINALIZADOR CAPILAR</t>
+          <t>HIDRAULICA</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n">
-        <v>7898961206721</v>
+        <v>7898197936010</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>SUPL ALIM OMEGA 3 HYPERNA 1UN (VDO)</t>
+          <t>SUPL ALIM OMEGA 3 NATUR 1UN (VDO)</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -9499,31 +9509,31 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>HIDRAULICA</t>
+          <t>PET FARMACIA</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">
-        <v>7898197936010</v>
+        <v>7898114063027</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>SUPL ALIM OMEGA 3 NATUR 1UN (VDO)</t>
+          <t>SUPL ALIM OMIX FERRO 525MG 70CPS (OMX)</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>VIDORA</t>
+          <t>ORIENT MIX</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>OMEGA 3 VDO</t>
+          <t>OMIX OMX</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
@@ -9547,31 +9557,31 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>PET FARMACIA</t>
+          <t>PEQUENO DOMESTICO</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n">
-        <v>7898114063027</v>
+        <v>7898722646759</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>SUPL ALIM OMIX FERRO 525MG 70CPS (OMX)</t>
+          <t>SUPL ALIM OTTIMA VITTA FERRO LINHA VERDE 1UN (NUS)</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ORIENT MIX</t>
+          <t>NATUS FARMA</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>OMIX OMX</t>
+          <t>OTTIMA VITTA NUS</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
@@ -9601,25 +9611,25 @@
     </row>
     <row r="188">
       <c r="A188" s="2" t="n">
-        <v>7898722646759</v>
+        <v>7898483535019</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>SUPL ALIM OTTIMA VITTA FERRO LINHA VERDE 1UN (NUS)</t>
+          <t>SUPL ALIM PHD MELATONINA GOTAS SAB MARACUJA 30ML (MAR)</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>NATUS FARMA</t>
+          <t>MARJAN FARMA</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>OTTIMA VITTA NUS</t>
+          <t>PHD MAR</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F188" t="inlineStr">
         <is>
@@ -9643,31 +9653,31 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>PEQUENO DOMESTICO</t>
+          <t>SHAMPOO</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n">
-        <v>7898483535019</v>
+        <v>7908277600325</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>SUPL ALIM PHD MELATONINA GOTAS SAB MARACUJA 30ML (MAR)</t>
+          <t>SUPL ALIM PICOLINATO CROMO 280MG 60UN (FAC)</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>MARJAN FARMA</t>
+          <t>FARMA CONDE</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>PHD MAR</t>
+          <t>PICOLINATO CROMO FAC</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F189" t="inlineStr">
         <is>
@@ -9691,17 +9701,17 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>SHAMPOO</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n">
-        <v>7908277600325</v>
+        <v>7898197933316</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>SUPL ALIM PICOLINATO CROMO 280MG 60UN (FAC)</t>
+          <t>SUPL ALIM PICOLINATO CROMO OTTIMA VIT 1UN (FAC)</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -9715,7 +9725,7 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F190" t="inlineStr">
         <is>
@@ -9739,31 +9749,31 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>SALGADO CONGELADO</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n">
-        <v>7898197933316</v>
+        <v>7898960179552</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>SUPL ALIM PICOLINATO CROMO OTTIMA VIT 1UN (FAC)</t>
+          <t>SUPL ALIM POWER SPIRULINA FITO 500MG 60CPS (PAG)</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>FARMA CONDE</t>
+          <t>PAGUE MENOS</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>PICOLINATO CROMO FAC</t>
+          <t>POWER PAG</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F191" t="inlineStr">
         <is>
@@ -9787,31 +9797,31 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>SALGADO CONGELADO</t>
+          <t>ACUCAR</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n">
-        <v>7898960179552</v>
+        <v>7898081730830</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>SUPL ALIM POWER SPIRULINA FITO 500MG 60CPS (PAG)</t>
+          <t>SUPL ALIM PRIMAVERA FARINHA MARACUJA 250MG 90CPS (PRU)</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>PAGUE MENOS</t>
+          <t>PRODUTOS PRIMAVERA</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>POWER PAG</t>
+          <t>PRIMAVERA PRU</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F192" t="inlineStr">
         <is>
@@ -9835,31 +9845,31 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>ACUCAR</t>
+          <t>FARINHA</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n">
-        <v>7898081730830</v>
+        <v>7898946434224</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>SUPL ALIM PRIMAVERA FARINHA MARACUJA 250MG 90CPS (PRU)</t>
+          <t>SUPL ALIM PRIMULA OLEO 1UN (PRP)</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>PRODUTOS PRIMAVERA</t>
+          <t>PRIMULA PAPEIS</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>PRIMAVERA PRU</t>
+          <t>PRIMULA PRP</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
@@ -9883,17 +9893,17 @@
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>FARINHA</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n">
-        <v>7898946434224</v>
+        <v>7898946435368</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>SUPL ALIM PRIMULA OLEO 1UN (PRP)</t>
+          <t>SUPL ALIM PRIMULA RAIA 1UN (PRP)</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -9931,31 +9941,31 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n">
-        <v>7898946435368</v>
+        <v>7898932877448</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>SUPL ALIM PRIMULA RAIA 1UN (PRP)</t>
+          <t>SUPL ALIM PROPOLIS APIARIO SEBASTIAO BALA MEL 38G (EXR)</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>PRIMULA PAPEIS</t>
+          <t>EXPRESSAO DA NATUREZA</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>PRIMULA PRP</t>
+          <t>PROPOLIS EXR</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="F195" t="inlineStr">
         <is>
@@ -9979,27 +9989,27 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>BALA E PIRULITO</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n">
-        <v>7898932877448</v>
+        <v>7898932877172</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>SUPL ALIM PROPOLIS APIARIO SEBASTIAO BALA MEL 38G (EXR)</t>
+          <t>SUPL ALIM PROPOLIS BALA DE GENGIBRE MEL FLORA 38G (NUS)</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>EXPRESSAO DA NATUREZA</t>
+          <t>NATUS FARMA</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>PROPOLIS EXR</t>
+          <t>PROPOLIS NUS</t>
         </is>
       </c>
       <c r="E196" t="n">
@@ -10033,25 +10043,25 @@
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
-        <v>7898932877172</v>
+        <v>7896663301348</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>SUPL ALIM PROPOLIS BALA DE GENGIBRE MEL FLORA 38G (NUS)</t>
+          <t>SUPL ALIM PROPOMAX 30CPS (AFL)</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>NATUS FARMA</t>
+          <t>APIS FLORA</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>PROPOLIS NUS</t>
+          <t>PROPOMAX AFL</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="F197" t="inlineStr">
         <is>
@@ -10075,27 +10085,27 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>BALA E PIRULITO</t>
+          <t>MEL</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n">
-        <v>7896663301348</v>
+        <v>7898638344251</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>SUPL ALIM PROPOMAX 30CPS (AFL)</t>
+          <t>SUPL ALIM QUALIVITA GRIPE FORTE 30CPRS (UNF)</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>APIS FLORA</t>
+          <t>UNIFABRA</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>PROPOMAX AFL</t>
+          <t>QUALIVITA UNF</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -10123,31 +10133,31 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>MEL</t>
+          <t>JARDINAGEM</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
-        <v>7898638344251</v>
+        <v>7899751213288</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>SUPL ALIM QUALIVITA GRIPE FORTE 30CPRS (UNF)</t>
+          <t>SUPL ALIM QVITA TRIPTOFANO 1000MG 60CPS (VNT)</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>UNIFABRA</t>
+          <t>VITAL PROD. NATURAIS LTDA</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>QUALIVITA UNF</t>
+          <t>QVITA VNT</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F199" t="inlineStr">
         <is>
@@ -10171,31 +10181,31 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>JARDINAGEM</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n">
-        <v>7899751213288</v>
+        <v>7898946435993</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>SUPL ALIM QVITA TRIPTOFANO 1000MG 60CPS (VNT)</t>
+          <t>SUPL ALIM RAIA 1000UI 30CPS (RDF)</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>VITAL PROD. NATURAIS LTDA</t>
+          <t>RAIA DROGASIL SA</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>QVITA VNT</t>
+          <t>RAIA RDF</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F200" t="inlineStr">
         <is>
@@ -10219,17 +10229,17 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>PAPELARIA OUTROS</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
-        <v>7898946435993</v>
+        <v>7898946435344</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA 1000UI 30CPS (RDF)</t>
+          <t>SUPL ALIM RAIA CAFEINA 1UN (RDF)</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -10243,7 +10253,7 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F201" t="inlineStr">
         <is>
@@ -10267,17 +10277,17 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>PAPELARIA OUTROS</t>
+          <t>VESTUARIO</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n">
-        <v>7898946435344</v>
+        <v>7898946435351</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA CAFEINA 1UN (RDF)</t>
+          <t>SUPL ALIM RAIA LINHACA 1UN (RDF)</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -10321,11 +10331,11 @@
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
-        <v>7898946435351</v>
+        <v>7898687730166</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA LINHACA 1UN (RDF)</t>
+          <t>SUPL ALIM RAIA OMEGA 3 1UN (RDF)</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -10363,13 +10373,13 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>VESTUARIO</t>
+          <t>PET ALIMENTO PARA AVE</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
-        <v>7898687730166</v>
+        <v>7898946435306</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -10411,17 +10421,17 @@
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>PET ALIMENTO PARA AVE</t>
+          <t>VESTUARIO</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n">
-        <v>7898946435306</v>
+        <v>7891066001413</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA OMEGA 3 1UN (RDF)</t>
+          <t>SUPL ALIM RAIA PICOLI CRO 60UN (RDF)</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -10435,7 +10445,7 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F205" t="inlineStr">
         <is>
@@ -10459,17 +10469,17 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>VESTUARIO</t>
+          <t>BRINQUEDO</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
-        <v>7891066001413</v>
+        <v>7891066001437</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA PICOLI CRO 60UN (RDF)</t>
+          <t>SUPL ALIM RAIA PROPOLVIT 60UN (RDF)</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -10507,17 +10517,17 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>BRINQUEDO</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n">
-        <v>7891066001437</v>
+        <v>7891066001475</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA PROPOLVIT 60UN (RDF)</t>
+          <t>SUPL ALIM RAIA VIT CDZ EFV 10UN (RDF)</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -10531,7 +10541,7 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="F207" t="inlineStr">
         <is>
@@ -10555,17 +10565,17 @@
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>PET ACESSORIO</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n">
-        <v>7891066001475</v>
+        <v>7891066001482</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA VIT CDZ EFV 10UN (RDF)</t>
+          <t>SUPL ALIM RAIA VIT CDZ EFV 30UN (RDF)</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -10579,7 +10589,7 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F208" t="inlineStr">
         <is>
@@ -10609,11 +10619,11 @@
     </row>
     <row r="209">
       <c r="A209" s="2" t="n">
-        <v>7891066001482</v>
+        <v>7896413896940</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA VIT CDZ EFV 30UN (RDF)</t>
+          <t>SUPL ALIM RAIA VIT CDZIN 1UN (RDF)</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -10627,7 +10637,7 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F209" t="inlineStr">
         <is>
@@ -10651,17 +10661,17 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>PET ACESSORIO</t>
+          <t>PAPELARIA OUTROS</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n">
-        <v>7896413896940</v>
+        <v>7891066005190</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA VIT CDZIN 1UN (RDF)</t>
+          <t>SUPL ALIM RAIA VIT CZINC 10UN (RDF)</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -10675,7 +10685,7 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F210" t="inlineStr">
         <is>
@@ -10699,17 +10709,17 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>PAPELARIA OUTROS</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n">
-        <v>7891066005190</v>
+        <v>7891066005213</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA VIT CZINC 10UN (RDF)</t>
+          <t>SUPL ALIM RAIA VIT CZINC 30UN (RDF)</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -10723,7 +10733,7 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F211" t="inlineStr">
         <is>
@@ -10753,11 +10763,11 @@
     </row>
     <row r="212">
       <c r="A212" s="2" t="n">
-        <v>7891066005213</v>
+        <v>7891066006463</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA VIT CZINC 30UN (RDF)</t>
+          <t>SUPL ALIM RAIA VITAMINA D 2000UI 1UN (RDF)</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -10771,7 +10781,7 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F212" t="inlineStr">
         <is>
@@ -10795,31 +10805,31 @@
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>CONSERVA VEGETAL</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n">
-        <v>7891066006463</v>
+        <v>7898074619081</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>SUPL ALIM RAIA VITAMINA D 2000UI 1UN (RDF)</t>
+          <t>SUPL ALIM REFORM DUO 7G (ZAM)</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>RAIA DROGASIL SA</t>
+          <t>ZAMBON</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>RAIA RDF</t>
+          <t>REFORM ZAM</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F213" t="inlineStr">
         <is>
@@ -10843,17 +10853,17 @@
       </c>
       <c r="L213" t="inlineStr">
         <is>
-          <t>CONSERVA VEGETAL</t>
+          <t>SUCO</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n">
-        <v>7898074619081</v>
+        <v>7898074616974</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>SUPL ALIM REFORM DUO 7G (ZAM)</t>
+          <t>SUPL ALIM REFORM MAX 3.5G (ZAM)</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -10867,7 +10877,7 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>7</v>
+        <v>3.5</v>
       </c>
       <c r="F214" t="inlineStr">
         <is>
@@ -10891,31 +10901,31 @@
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t>SUCO</t>
+          <t>ELETRODOMESTICO</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n">
-        <v>7898074616974</v>
+        <v>7899640801169</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>SUPL ALIM REFORM MAX 3.5G (ZAM)</t>
+          <t>SUPL ALIM REGULARE 10X5G (MOM)</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>ZAMBON</t>
+          <t>MOMENTA FARMA</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>REFORM ZAM</t>
+          <t>REGULARE MOM</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>3.5</v>
+        <v>50</v>
       </c>
       <c r="F215" t="inlineStr">
         <is>
@@ -10932,6 +10942,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I215" s="4" t="inlineStr">
+        <is>
+          <t>CRIAR MARCA</t>
+        </is>
+      </c>
       <c r="K215" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -10939,31 +10954,31 @@
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t>ELETRODOMESTICO</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n">
-        <v>7899640801169</v>
+        <v>7898704671434</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>SUPL ALIM REGULARE 10X5G (MOM)</t>
+          <t>SUPL ALIM SEMPRE FINA SHAPE VITAMINA A 550MG 60CPS (VPR)</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>MOMENTA FARMA</t>
+          <t>VITA PREMIUM</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>REGULARE MOM</t>
+          <t>SEMPRE VPR</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F216" t="inlineStr">
         <is>
@@ -10980,11 +10995,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I216" s="4" t="inlineStr">
-        <is>
-          <t>CRIAR MARCA</t>
-        </is>
-      </c>
       <c r="K216" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -10992,31 +11002,31 @@
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>LEGUME</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n">
-        <v>7898704671434</v>
+        <v>7896083411818</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>SUPL ALIM SEMPRE FINA SHAPE VITAMINA A 550MG 60CPS (VPR)</t>
+          <t>SUPL ALIM SIMPLI 1000UI 20ML (HER)</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>VITA PREMIUM</t>
+          <t>HERBARIUM</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>SEMPRE VPR</t>
+          <t>SIMPLI HER</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="F217" t="inlineStr">
         <is>
@@ -11033,6 +11043,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I217" s="4" t="inlineStr">
+        <is>
+          <t>CRIAR MARCA</t>
+        </is>
+      </c>
       <c r="K217" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -11040,31 +11055,31 @@
       </c>
       <c r="L217" t="inlineStr">
         <is>
-          <t>LEGUME</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n">
-        <v>7896083411818</v>
+        <v>7896658035616</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>SUPL ALIM SIMPLI 1000UI 20ML (HER)</t>
+          <t>SUPL ALIM SITOL 200MCG 21G (ACH)</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>HERBARIUM</t>
+          <t>ACHE LABORATORIOS FARMACEUTICOS SA</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>SIMPLI HER</t>
+          <t>SITOL ACH</t>
         </is>
       </c>
       <c r="E218" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F218" t="inlineStr">
         <is>
@@ -11093,13 +11108,13 @@
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>JARDINAGEM</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n">
-        <v>7896658035616</v>
+        <v>7896658035623</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -11146,31 +11161,31 @@
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>JARDINAGEM</t>
+          <t>MATERIAL OUTROS</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n">
-        <v>7896658035623</v>
+        <v>7898664817613</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>SUPL ALIM SITOL 200MCG 21G (ACH)</t>
+          <t>SUPL ALIM SMART LIFE IOIMBINA 500.0MG 60CPS (SMA)</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>ACHE LABORATORIOS FARMACEUTICOS SA</t>
+          <t>SMART LIFE</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>SITOL ACH</t>
+          <t>SMART LIFE SMA</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="F220" t="inlineStr">
         <is>
@@ -11187,11 +11202,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I220" s="4" t="inlineStr">
-        <is>
-          <t>CRIAR MARCA</t>
-        </is>
-      </c>
       <c r="K220" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -11199,27 +11209,27 @@
       </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>MATERIAL OUTROS</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n">
-        <v>7898664817613</v>
+        <v>7898197931701</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>SUPL ALIM SMART LIFE IOIMBINA 500.0MG 60CPS (SMA)</t>
+          <t>SUPL ALIM SOFTGEL OLEO DE ABACATE 1000MG 60CPS (MEF)</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>SMART LIFE</t>
+          <t>MELFORT</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>SMART LIFE SMA</t>
+          <t>SOFTGEL MEF</t>
         </is>
       </c>
       <c r="E221" t="n">
@@ -11247,31 +11257,31 @@
       </c>
       <c r="L221" t="inlineStr">
         <is>
-          <t>SUPLEMENTO PARA ACADEMIA</t>
+          <t>FINALIZADOR CAPILAR</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n">
-        <v>7898197931701</v>
+        <v>7898568950829</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>SUPL ALIM SOFTGEL OLEO DE ABACATE 1000MG 60CPS (MEF)</t>
+          <t>SUPL ALIM SPIRRO CANELA DE VELHO 500MG 500ML (SPI)</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>MELFORT</t>
+          <t>SPIRRO</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>SOFTGEL MEF</t>
+          <t>SPIRRO SPI</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>60</v>
+        <v>500</v>
       </c>
       <c r="F222" t="inlineStr">
         <is>
@@ -11295,31 +11305,31 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>FINALIZADOR CAPILAR</t>
+          <t>ACESSORIO COZINHA</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n">
-        <v>7898568950829</v>
+        <v>7898142064522</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>SUPL ALIM SPIRRO CANELA DE VELHO 500MG 500ML (SPI)</t>
+          <t>SUPL ALIM SPIRULINA FAZ 50G (POY)</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>SPIRRO</t>
+          <t>POYTARA</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>SPIRRO SPI</t>
+          <t>SPIRULINA POY</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="F223" t="inlineStr">
         <is>
@@ -11343,31 +11353,31 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>ACESSORIO COZINHA</t>
+          <t>BRINQUEDO</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n">
-        <v>7898142064522</v>
+        <v>30768038199</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>SUPL ALIM SPIRULINA FAZ 50G (POY)</t>
+          <t>SUPL ALIM SUNDOWN OMEGA 3 1000MG 60CPS (NES)</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>POYTARA</t>
+          <t>NESTLE CIA</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>SPIRULINA POY</t>
+          <t>SUNDOWN NES</t>
         </is>
       </c>
       <c r="E224" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F224" t="inlineStr">
         <is>
@@ -11391,17 +11401,17 @@
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t>BRINQUEDO</t>
+          <t>TRATAMENTO FACIAL</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n">
-        <v>30768038199</v>
+        <v>30768358631</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>SUPL ALIM SUNDOWN OMEGA 3 1000MG 60CPS (NES)</t>
+          <t>SUPL ALIM SUNDOWN SELENIO 34MG 60UN (NES)</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -11439,27 +11449,27 @@
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>TRATAMENTO FACIAL</t>
+          <t>PET LIMPEZA</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n">
-        <v>30768358631</v>
+        <v>7898743919702</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>SUPL ALIM SUNDOWN SELENIO 34MG 60UN (NES)</t>
+          <t>SUPL ALIM SUNFOOD MOROSEK 2000MG 60CPS</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>NESTLE CIA</t>
+          <t>OUTRO FABRICANTE</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>SUNDOWN NES</t>
+          <t>SUNFOOD</t>
         </is>
       </c>
       <c r="E226" t="n">
@@ -11480,6 +11490,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I226" s="4" t="inlineStr">
+        <is>
+          <t>SEM FABRICANTE</t>
+        </is>
+      </c>
       <c r="K226" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -11487,31 +11502,31 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>PET LIMPEZA</t>
+          <t>LEGUME</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n">
-        <v>7898743919702</v>
+        <v>7897551700380</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>SUPL ALIM SUNFOOD MOROSEK 2000MG 60CPS</t>
+          <t>SUPL ALIM SUPERMEL GELEIA REAL LIOFILIZADO 700MG 45CPS (SPP)</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>SUPERMEL</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>SUNFOOD</t>
+          <t>SUPERMEL SPP</t>
         </is>
       </c>
       <c r="E227" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F227" t="inlineStr">
         <is>
@@ -11528,11 +11543,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I227" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
-        </is>
-      </c>
       <c r="K227" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -11540,31 +11550,31 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>LEGUME</t>
+          <t>GELEIA OUTROS</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n">
-        <v>7897551700380</v>
+        <v>7898572401003</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>SUPL ALIM SUPERMEL GELEIA REAL LIOFILIZADO 700MG 45CPS (SPP)</t>
+          <t>SUPL ALIM SUPLAN UXI AMARELO UNHA DE GATO MELHOR 60CPS (ASP)</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>SUPERMEL</t>
+          <t>ASPEN</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>SUPERMEL SPP</t>
+          <t>SUPLAN ASP</t>
         </is>
       </c>
       <c r="E228" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="F228" t="inlineStr">
         <is>
@@ -11588,27 +11598,27 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>GELEIA OUTROS</t>
+          <t>MOLHO</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n">
-        <v>7898572401003</v>
+        <v>7898411817491</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>SUPL ALIM SUPLAN UXI AMARELO UNHA DE GATO MELHOR 60CPS (ASP)</t>
+          <t>SUPL ALIM TAKECARE OLEO COCO 1000MG 60CPS (TKC)</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>ASPEN</t>
+          <t>TAKE CARE IND</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>SUPLAN ASP</t>
+          <t>TAKECARE TKC</t>
         </is>
       </c>
       <c r="E229" t="n">
@@ -11636,31 +11646,31 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>MOLHO</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n">
-        <v>7898411817491</v>
+        <v>742832585248</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>SUPL ALIM TAKECARE OLEO COCO 1000MG 60CPS (TKC)</t>
+          <t>SUPL ALIM TERRA MAIS MAGNOCALCIO 500MG 120CPS (TEA)</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>TAKE CARE IND</t>
+          <t>TERRA MAIS</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>TAKECARE TKC</t>
+          <t>TERRA MAIS TEA</t>
         </is>
       </c>
       <c r="E230" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F230" t="inlineStr">
         <is>
@@ -11684,17 +11694,17 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>JARDINAGEM</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n">
-        <v>742832585248</v>
+        <v>7891197885395</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>SUPL ALIM TERRA MAIS MAGNOCALCIO 500MG 120CPS (TEA)</t>
+          <t>SUPL ALIM TERRA MAIS OLEO LINHACA 500MG 60CPS (TEA)</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -11708,7 +11718,7 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F231" t="inlineStr">
         <is>
@@ -11732,31 +11742,31 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>JARDINAGEM</t>
+          <t>CONSERVA VEGETAL</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n">
-        <v>7891197885395</v>
+        <v>7898171780400</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>SUPL ALIM TERRA MAIS OLEO LINHACA 500MG 60CPS (TEA)</t>
+          <t>SUPL ALIM TIARAJU OLEO ALHO 500MG 70CPS (TIR)</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>TERRA MAIS</t>
+          <t>TIARAJU</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>TERRA MAIS TEA</t>
+          <t>TIARAJU TIR</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
@@ -11780,31 +11790,31 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>CONSERVA VEGETAL</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n">
-        <v>7898171780400</v>
+        <v>618341417403</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>SUPL ALIM TIARAJU OLEO ALHO 500MG 70CPS (TIR)</t>
+          <t>SUPL ALIM TRIPTOFANO 30CPRS</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>TIARAJU</t>
+          <t>OUTRO FABRICANTE</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>TIARAJU TIR</t>
+          <t>TRIPTOFANO</t>
         </is>
       </c>
       <c r="E233" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F233" t="inlineStr">
         <is>
@@ -11821,6 +11831,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I233" s="4" t="inlineStr">
+        <is>
+          <t>SEM FABRICANTE</t>
+        </is>
+      </c>
       <c r="K233" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -11828,17 +11843,17 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>PET FARMACIA</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n">
-        <v>618341417403</v>
+        <v>7898005960077</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>SUPL ALIM TRIPTOFANO 30CPRS</t>
+          <t>SUPL ALIM TURUNA CHA VERDE 70G</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -11848,11 +11863,11 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>TRIPTOFANO</t>
+          <t>TURUNA</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="F234" t="inlineStr">
         <is>
@@ -11881,17 +11896,17 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>PET FARMACIA</t>
+          <t>CHA PRONTO</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n">
-        <v>7898005960077</v>
+        <v>7898716067348</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>SUPL ALIM TURUNA CHA VERDE 70G</t>
+          <t>SUPL ALIM ULTRA MAGNEO FORCE LIBERACAO 60CPS</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -11901,11 +11916,11 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>TURUNA</t>
+          <t>OUTRA MARCA</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F235" t="inlineStr">
         <is>
@@ -11934,31 +11949,31 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>CHA PRONTO</t>
+          <t>TRATAMENTO CAPILAR</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n">
-        <v>7898716067348</v>
+        <v>7896023749087</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>SUPL ALIM ULTRA MAGNEO FORCE LIBERACAO 60CPS</t>
+          <t>SUPL ALIM UP VITAM 2000UI 10ML (CAT)</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>CATARINENSE PHARMA</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>OUTRA MARCA</t>
+          <t>UP VITAM CAT</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="F236" t="inlineStr">
         <is>
@@ -11973,11 +11988,6 @@
       <c r="H236" t="inlineStr">
         <is>
           <t>Sem indícios de CI</t>
-        </is>
-      </c>
-      <c r="I236" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
         </is>
       </c>
       <c r="K236" s="3" t="inlineStr">
@@ -11993,25 +12003,25 @@
     </row>
     <row r="237">
       <c r="A237" s="2" t="n">
-        <v>7896023749087</v>
+        <v>7898965555108</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>SUPL ALIM UP VITAM 2000UI 10ML (CAT)</t>
+          <t>SUPL ALIM V HAPPY OMEGA 3 120CPS (DRV)</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>CATARINENSE PHARMA</t>
+          <t>DROGARIA VENANCIO</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>UP VITAM CAT</t>
+          <t>V HAPPY DRV</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="F237" t="inlineStr">
         <is>
@@ -12035,31 +12045,31 @@
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t>TRATAMENTO CAPILAR</t>
+          <t>VINHO</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n">
-        <v>7898965555108</v>
+        <v>7899558303083</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>SUPL ALIM V HAPPY OMEGA 3 120CPS (DRV)</t>
+          <t>SUPL ALIM VIA TERRA OLEO DE COCO 60CPS (VIE)</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>DROGARIA VENANCIO</t>
+          <t>VIA TERRA PRODUTOS NATURAIS</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>V HAPPY DRV</t>
+          <t>VIA TERRA VIE</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F238" t="inlineStr">
         <is>
@@ -12083,31 +12093,31 @@
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>VINHO</t>
+          <t>OLEO</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n">
-        <v>7899558303083</v>
+        <v>7898906170193</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>SUPL ALIM VIA TERRA OLEO DE COCO 60CPS (VIE)</t>
+          <t>SUPL ALIM VILLAGE OLEO CARTAMO COCO 1000MG 1G (VIC)</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>VIA TERRA PRODUTOS NATURAIS</t>
+          <t>VILLAGE CEPAM</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>VIA TERRA VIE</t>
+          <t>VILLAGE VIC</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="F239" t="inlineStr">
         <is>
@@ -12137,11 +12147,11 @@
     </row>
     <row r="240">
       <c r="A240" s="2" t="n">
-        <v>7898906170193</v>
+        <v>7898906169869</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>SUPL ALIM VILLAGE OLEO CARTAMO COCO 1000MG 1G (VIC)</t>
+          <t>SUPL ALIM VILLAGE OLEO DE COCO VILA 1000MG 120CPS (VIC)</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -12155,7 +12165,7 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="F240" t="inlineStr">
         <is>
@@ -12179,31 +12189,31 @@
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>OLEO</t>
+          <t>FINALIZADOR CAPILAR</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n">
-        <v>7898906169869</v>
+        <v>7897642733174</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>SUPL ALIM VILLAGE OLEO DE COCO VILA 1000MG 120CPS (VIC)</t>
+          <t>SUPL ALIM VINAGRE DE MACA 500MG 60CPS (NNC)</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>VILLAGE CEPAM</t>
+          <t>NATUNECTAR</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>VILLAGE VIC</t>
+          <t>VINAGRE DE MACA NNC</t>
         </is>
       </c>
       <c r="E241" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F241" t="inlineStr">
         <is>
@@ -12227,31 +12237,31 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>FINALIZADOR CAPILAR</t>
+          <t>VINAGRE</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n">
-        <v>7897642733174</v>
+        <v>7891066001499</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>SUPL ALIM VINAGRE DE MACA 500MG 60CPS (NNC)</t>
+          <t>SUPL ALIM VIT DROG CDZ EFV 10UN (ALL)</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>NATUNECTAR</t>
+          <t>VIT</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>VINAGRE DE MACA NNC</t>
+          <t>VIT ALL</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="F242" t="inlineStr">
         <is>
@@ -12275,17 +12285,17 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>VINAGRE</t>
+          <t>PET ACESSORIO</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n">
-        <v>7891066001499</v>
+        <v>7891066001505</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>SUPL ALIM VIT DROG CDZ EFV 10UN (ALL)</t>
+          <t>SUPL ALIM VIT DROG CDZ EFV 30UN (ALL)</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -12299,7 +12309,7 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F243" t="inlineStr">
         <is>
@@ -12329,11 +12339,11 @@
     </row>
     <row r="244">
       <c r="A244" s="2" t="n">
-        <v>7891066001505</v>
+        <v>30768504144</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>SUPL ALIM VIT DROG CDZ EFV 30UN (ALL)</t>
+          <t>SUPL ALIM VIT E SUND VITAMINA MIXED 180UN (VTT)</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -12343,11 +12353,11 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>VIT ALL</t>
+          <t>VIT E VTT</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="F244" t="inlineStr">
         <is>
@@ -12371,31 +12381,31 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>PET ACESSORIO</t>
+          <t>CODIGO INTERNO</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n">
-        <v>30768504144</v>
+        <v>7898766590544</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>SUPL ALIM VIT E SUND VITAMINA MIXED 180UN (VTT)</t>
+          <t>SUPL ALIM VITA VINAGRE DE MACA GOMAS 30CPRS (VPR)</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>VIT</t>
+          <t>VITA PREMIUM</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>VIT E VTT</t>
+          <t>VITA VPR</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="F245" t="inlineStr">
         <is>
@@ -12419,27 +12429,27 @@
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>CODIGO INTERNO</t>
+          <t>VINAGRE</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n">
-        <v>7898766590544</v>
+        <v>7908041910995</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>SUPL ALIM VITA VINAGRE DE MACA GOMAS 30CPRS (VPR)</t>
+          <t>SUPL ALIM VITAMINA E OLEO SEMENTE ABOB GOTAS 30ML (FLN)</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>VITA PREMIUM</t>
+          <t>FLORA NATIVA DO BRASIL</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>VITA VPR</t>
+          <t>VITAMINA E FLN</t>
         </is>
       </c>
       <c r="E246" t="n">
@@ -12467,31 +12477,31 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>VINAGRE</t>
+          <t>FINALIZADOR CAPILAR</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n">
-        <v>7908041910995</v>
+        <v>7898994538714</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>SUPL ALIM VITAMINA E OLEO SEMENTE ABOB GOTAS 30ML (FLN)</t>
+          <t>SUPL ALIM VITAMINAS 1000MG 1UN (MXR)</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>FLORA NATIVA DO BRASIL</t>
+          <t>MAXINUTRI</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>VITAMINA E FLN</t>
+          <t>VITAMINAS MXR</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F247" t="inlineStr">
         <is>
@@ -12515,7 +12525,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>FINALIZADOR CAPILAR</t>
+          <t>SUPLEMENTO PARA ACADEMIA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Farmácia: sigla obrigatória (fabricante pela marca nas bases; genérico sem dono vira OUTRA MARCA; marca sem dono vira o próprio fabricante; sigla gerada sempre com 3 caracteres)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ymBuSrNzAQRN5kGJoFo1p
</commit_message>
<xml_diff>
--- a/classificador/dados/vitamina_mineral_500_classificado.xlsx
+++ b/classificador/dados/vitamina_mineral_500_classificado.xlsx
@@ -2266,25 +2266,25 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>7898946435184</v>
+        <v>7898332900296</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DROGASIL CALCIOD 1UN (RDF)</t>
+          <t>DOLOMITA NATURA LIFE COMPL MINERAL 200G (SUP)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AURAQUIMICA</t>
+          <t>SUP</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>DROGASIL RDF</t>
+          <t>SUP SUP</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2301,6 +2301,11 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>CRIAR FABRICANTE</t>
+        </is>
+      </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -2308,31 +2313,31 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>BALA E PIRULITO</t>
+          <t>PET ALIMENTO PARA AVE</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>7896658029523</v>
+        <v>7898946435184</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>INELATTE ACHEVITA INELLATE CHOCOLATE TABS MAST 30UN (TAB)</t>
+          <t>DROGASIL CALCIOD 1UN (RDF)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ACHE LABORATORIOS FARMACEUTICOS SA</t>
+          <t>AURAQUIMICA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>INELATTE TAB</t>
+          <t>DROGASIL RDF</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2356,17 +2361,17 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>CHOCOLATE</t>
+          <t>BALA E PIRULITO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>7896658033209</v>
+        <v>7896658029523</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>INELATTE CHOCOLATE 60UN (ACH)</t>
+          <t>INELATTE ACHEVITA INELLATE CHOCOLATE TABS MAST 30UN (TAB)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2376,11 +2381,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>INELATTE ACH</t>
+          <t>INELATTE TAB</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2410,11 +2415,11 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>7896658033162</v>
+        <v>7896658033209</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>INELATTE CHOCOLATE TABL 30UN (TAB)</t>
+          <t>INELATTE CHOCOLATE 60UN (ACH)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2424,11 +2429,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>INELATTE TAB</t>
+          <t>INELATTE ACH</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2452,31 +2457,31 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>SOBREMESA PRONTA GELIFICADA</t>
+          <t>CHOCOLATE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>7891058020576</v>
+        <v>7896658033162</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>OSCAL CIT 500MG 30X3G (C30)</t>
+          <t>INELATTE CHOCOLATE TABL 30UN (TAB)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SANOFI FARMACEUTICA</t>
+          <t>ACHE LABORATORIOS FARMACEUTICOS SA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>OSCAL C30</t>
+          <t>INELATTE TAB</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2500,17 +2505,17 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>PET ALIMENTO PARA GATO</t>
+          <t>SOBREMESA PRONTA GELIFICADA</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>7891058018573</v>
+        <v>7891058020576</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>OSCAL KIDS SUSPENSAO 150ML (SNF)</t>
+          <t>OSCAL CIT 500MG 30X3G (C30)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2520,11 +2525,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>OSCAL SNF</t>
+          <t>OSCAL C30</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2548,31 +2553,31 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>ESCOVA DENTAL</t>
+          <t>PET ALIMENTO PARA GATO</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>7898279422202</v>
+        <v>7891058018573</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PRADOCALCIO 1L (PAA)</t>
+          <t>OSCAL KIDS SUSPENSAO 150ML (SNF)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LABORATORIO PRADO</t>
+          <t>SANOFI FARMACEUTICA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>PRADOCALCIO PAA</t>
+          <t>OSCAL SNF</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1000</v>
+        <v>150</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2596,31 +2601,31 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>ACESSORIO CASA</t>
+          <t>ESCOVA DENTAL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>7898332900296</v>
+        <v>7898279422202</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SUP DOLOMITA NATURA LIFE COMPL MINERAL 200G</t>
+          <t>PRADOCALCIO 1L (PAA)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>LABORATORIO PRADO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SUP</t>
+          <t>PRADOCALCIO PAA</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2637,11 +2642,6 @@
           <t>Sem indícios de CI</t>
         </is>
       </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
-        </is>
-      </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>PET ALIMENTO PARA AVE</t>
+          <t>ACESSORIO CASA</t>
         </is>
       </c>
     </row>
@@ -3432,17 +3432,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GLUCOSAMIMA CONDROITINA 30UN</t>
+          <t>GLUCOSAMIMA CONDROITINA 30UN (GLU)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>GLUCOSAMIMA</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>GLUCOSAMIMA</t>
+          <t>GLUCOSAMIMA GLU</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>CRIAR MARCA; SEM FABRICANTE</t>
+          <t>CRIAR MARCA E FABRICANTE</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
@@ -3485,17 +3485,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>OCEAN TERMOMETRO 1UN</t>
+          <t>OCEAN TERMOMETRO 1UN (OCE)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>OCEAN</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>OCEAN</t>
+          <t>OCEAN OCE</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -3514,11 +3514,6 @@
       <c r="H63" t="inlineStr">
         <is>
           <t>Sem indícios de CI</t>
-        </is>
-      </c>
-      <c r="I63" s="4" t="inlineStr">
-        <is>
-          <t>SEM FABRICANTE</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
@@ -3985,17 +3980,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SUPL ALIM MULT CONTROL PLUS A Z 60UN</t>
+          <t>SUPL ALIM MULT CONTROL PLUS A Z 60UN (CON)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>CONTROL</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>CONTROL</t>
+          <t>CONTROL CON</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -4018,7 +4013,7 @@
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>SEM FABRICANTE</t>
+          <t>CRIAR FABRICANTE</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
@@ -4768,17 +4763,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SUPL ALIM MULT HAIR UP GOMAS EKB 30UN</t>
+          <t>SUPL ALIM MULT HAIR UP GOMAS EKB 30UN (HAI)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>HAIR UP</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>HAIR UP</t>
+          <t>HAIR UP HAI</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -4801,7 +4796,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>SEM FABRICANTE</t>
+          <t>CRIAR FABRICANTE</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
@@ -5359,17 +5354,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SUPL ALIM MULT PHARMALIV MULTI A Z CABELOS UNH 1UN</t>
+          <t>SUPL ALIM MULT PHARMALIV MULTI A Z CABELOS UNH 1UN (PHA)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>PHARMALIV</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>PHARMALIV</t>
+          <t>PHARMALIV PHA</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -5392,7 +5387,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>SEM FABRICANTE</t>
+          <t>CRIAR FABRICANTE</t>
         </is>
       </c>
       <c r="K101" s="3" t="inlineStr">
@@ -8092,17 +8087,17 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>SUPL ALIM JIANG HUANG MTC 700.0MG 120CPS</t>
+          <t>SUPL ALIM JIANG HUANG MTC 700.0MG 120CPS (JIA)</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>JIANG HUANG</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>JIANG HUANG</t>
+          <t>JIANG HUANG JIA</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -8125,7 +8120,7 @@
       </c>
       <c r="I157" s="4" t="inlineStr">
         <is>
-          <t>SEM FABRICANTE</t>
+          <t>CRIAR FABRICANTE</t>
         </is>
       </c>
       <c r="K157" s="3" t="inlineStr">
@@ -11459,17 +11454,17 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>SUPL ALIM SUNFOOD MOROSEK 2000MG 60CPS</t>
+          <t>SUPL ALIM SUNFOOD MOROSEK 2000MG 60CPS (SUN)</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>SUNFOOD</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>SUNFOOD</t>
+          <t>SUNFOOD SUN</t>
         </is>
       </c>
       <c r="E226" t="n">
@@ -11492,7 +11487,7 @@
       </c>
       <c r="I226" s="4" t="inlineStr">
         <is>
-          <t>SEM FABRICANTE</t>
+          <t>CRIAR FABRICANTE</t>
         </is>
       </c>
       <c r="K226" s="3" t="inlineStr">
@@ -11810,7 +11805,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>TRIPTOFANO</t>
+          <t>OUTRA MARCA</t>
         </is>
       </c>
       <c r="E233" t="n">
@@ -11853,17 +11848,17 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>SUPL ALIM TURUNA CHA VERDE 70G</t>
+          <t>SUPL ALIM TURUNA CHA VERDE 70G (TUR)</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>TURUNA</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>TURUNA</t>
+          <t>TURUNA TUR</t>
         </is>
       </c>
       <c r="E234" t="n">
@@ -11886,7 +11881,7 @@
       </c>
       <c r="I234" s="4" t="inlineStr">
         <is>
-          <t>SEM FABRICANTE</t>
+          <t>CRIAR FABRICANTE</t>
         </is>
       </c>
       <c r="K234" s="3" t="inlineStr">
@@ -12891,17 +12886,17 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>SUPL ALIM ZANOTTI OLEO DE COCO 60CPS</t>
+          <t>SUPL ALIM ZANOTTI OLEO DE COCO 60CPS (ZAN)</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>OUTRO FABRICANTE</t>
+          <t>ZANOTTI</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>ZANOTTI</t>
+          <t>ZANOTTI ZAN</t>
         </is>
       </c>
       <c r="E255" t="n">
@@ -12924,7 +12919,7 @@
       </c>
       <c r="I255" s="4" t="inlineStr">
         <is>
-          <t>SEM FABRICANTE</t>
+          <t>CRIAR FABRICANTE</t>
         </is>
       </c>
       <c r="K255" s="3" t="inlineStr">
@@ -23431,7 +23426,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>PVPI RIODEINE ALTOMOTOLIA 1UN</t>
+          <t>PVPI RIODEINE ALTOMOTOLIA 1UN (PVP)</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">

</xml_diff>